<commit_message>
county field in workplace
</commit_message>
<xml_diff>
--- a/bcse_site/bcse_app/static/xls/WorkPlaceTemplate.xlsx
+++ b/bcse_site/bcse_app/static/xls/WorkPlaceTemplate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10708"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snp146/Documents/BCSE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snp146/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033AECD9-E90E-8E4E-93CF-3E62A91AFD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F592D115-6AD4-9F4B-B399-31308D2B82F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2420" windowWidth="28040" windowHeight="17440" xr2:uid="{B5201E93-1EAE-7D4F-AF55-CCC0B5A3E04D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>School</t>
   </si>
@@ -369,6 +369,43 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <r>
+      <t>County(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>Cook</t>
+  </si>
+  <si>
+    <t>Lake</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -431,11 +468,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -455,9 +491,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -495,7 +531,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -601,7 +637,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -743,7 +779,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -751,17 +787,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AE7D386-0738-944D-BD9A-00E3C44559D0}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.1640625" customWidth="1"/>
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
@@ -781,9 +817,12 @@
         <v>63</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
@@ -791,7 +830,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6DFF9AAD-2E72-BE48-AA42-3D79C6FC15A7}">
           <x14:formula1>
             <xm:f>Options!$A$2:$A$3</xm:f>
@@ -801,6 +840,12 @@
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{31BB5CC4-3820-774C-BBBE-945E58C4311F}">
           <x14:formula1>
             <xm:f>Options!$B$2:$B$56</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{003C4A26-952C-FE4C-9620-88B68ED45AA9}">
+          <x14:formula1>
+            <xm:f>Options!$C$2:$C$4</xm:f>
           </x14:formula1>
           <xm:sqref>G2:G1048576</xm:sqref>
         </x14:dataValidation>
@@ -816,7 +861,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="13.1640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -826,13 +871,19 @@
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="2" spans="1:6" ht="20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -842,23 +893,29 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>70</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>71</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="2"/>
@@ -866,7 +923,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="2"/>
@@ -874,7 +931,7 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="2"/>
@@ -882,7 +939,7 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="2"/>
@@ -890,7 +947,7 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2"/>
@@ -898,7 +955,7 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="2"/>
@@ -906,7 +963,7 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="2"/>
@@ -914,7 +971,7 @@
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D12" s="2"/>
@@ -922,7 +979,7 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D13" s="2"/>
@@ -930,7 +987,7 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="2"/>
@@ -938,7 +995,7 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="2"/>
@@ -946,7 +1003,7 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="2"/>
@@ -954,7 +1011,7 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="2"/>
@@ -962,7 +1019,7 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="2"/>
@@ -970,7 +1027,7 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D19" s="2"/>
@@ -978,7 +1035,7 @@
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="2"/>
@@ -986,7 +1043,7 @@
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D21" s="2"/>
@@ -994,7 +1051,7 @@
       <c r="F21" s="2"/>
     </row>
     <row r="22" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D22" s="2"/>
@@ -1002,7 +1059,7 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D23" s="2"/>
@@ -1010,7 +1067,7 @@
       <c r="F23" s="2"/>
     </row>
     <row r="24" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D24" s="2"/>
@@ -1018,7 +1075,7 @@
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D25" s="2"/>
@@ -1026,7 +1083,7 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="2"/>
@@ -1034,7 +1091,7 @@
       <c r="F26" s="2"/>
     </row>
     <row r="27" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D27" s="2"/>
@@ -1042,7 +1099,7 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>29</v>
       </c>
       <c r="D28" s="2"/>
@@ -1050,7 +1107,7 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>30</v>
       </c>
       <c r="D29" s="2"/>
@@ -1058,7 +1115,7 @@
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>31</v>
       </c>
       <c r="D30" s="2"/>
@@ -1066,7 +1123,7 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D31" s="2"/>
@@ -1074,7 +1131,7 @@
       <c r="F31" s="2"/>
     </row>
     <row r="32" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D32" s="2"/>
@@ -1082,7 +1139,7 @@
       <c r="F32" s="2"/>
     </row>
     <row r="33" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D33" s="2"/>
@@ -1090,7 +1147,7 @@
       <c r="F33" s="2"/>
     </row>
     <row r="34" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>35</v>
       </c>
       <c r="D34" s="2"/>
@@ -1098,7 +1155,7 @@
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>36</v>
       </c>
       <c r="D35" s="2"/>
@@ -1106,7 +1163,7 @@
       <c r="F35" s="2"/>
     </row>
     <row r="36" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D36" s="2"/>
@@ -1114,7 +1171,7 @@
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>38</v>
       </c>
       <c r="D37" s="2"/>
@@ -1122,7 +1179,7 @@
       <c r="F37" s="2"/>
     </row>
     <row r="38" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="3" t="s">
         <v>39</v>
       </c>
       <c r="D38" s="2"/>
@@ -1130,7 +1187,7 @@
       <c r="F38" s="2"/>
     </row>
     <row r="39" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D39" s="2"/>
@@ -1138,7 +1195,7 @@
       <c r="F39" s="2"/>
     </row>
     <row r="40" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="3" t="s">
         <v>41</v>
       </c>
       <c r="D40" s="2"/>
@@ -1146,7 +1203,7 @@
       <c r="F40" s="2"/>
     </row>
     <row r="41" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D41" s="2"/>
@@ -1154,7 +1211,7 @@
       <c r="F41" s="2"/>
     </row>
     <row r="42" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D42" s="2"/>
@@ -1162,7 +1219,7 @@
       <c r="F42" s="2"/>
     </row>
     <row r="43" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="3" t="s">
         <v>44</v>
       </c>
       <c r="D43" s="2"/>
@@ -1170,7 +1227,7 @@
       <c r="F43" s="2"/>
     </row>
     <row r="44" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D44" s="2"/>
@@ -1178,7 +1235,7 @@
       <c r="F44" s="2"/>
     </row>
     <row r="45" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>46</v>
       </c>
       <c r="D45" s="2"/>
@@ -1186,7 +1243,7 @@
       <c r="F45" s="2"/>
     </row>
     <row r="46" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D46" s="2"/>
@@ -1194,7 +1251,7 @@
       <c r="F46" s="2"/>
     </row>
     <row r="47" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>48</v>
       </c>
       <c r="D47" s="2"/>
@@ -1202,7 +1259,7 @@
       <c r="F47" s="2"/>
     </row>
     <row r="48" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D48" s="2"/>
@@ -1210,7 +1267,7 @@
       <c r="F48" s="2"/>
     </row>
     <row r="49" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D49" s="2"/>
@@ -1218,7 +1275,7 @@
       <c r="F49" s="2"/>
     </row>
     <row r="50" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D50" s="2"/>
@@ -1226,7 +1283,7 @@
       <c r="F50" s="2"/>
     </row>
     <row r="51" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D51" s="2"/>
@@ -1234,7 +1291,7 @@
       <c r="F51" s="2"/>
     </row>
     <row r="52" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D52" s="2"/>
@@ -1242,7 +1299,7 @@
       <c r="F52" s="2"/>
     </row>
     <row r="53" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D53" s="2"/>
@@ -1250,7 +1307,7 @@
       <c r="F53" s="2"/>
     </row>
     <row r="54" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="3" t="s">
         <v>55</v>
       </c>
       <c r="D54" s="2"/>
@@ -1258,7 +1315,7 @@
       <c r="F54" s="2"/>
     </row>
     <row r="55" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D55" s="2"/>
@@ -1266,7 +1323,7 @@
       <c r="F55" s="2"/>
     </row>
     <row r="56" spans="2:6" ht="20" x14ac:dyDescent="0.2">
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="3" t="s">
         <v>57</v>
       </c>
       <c r="D56" s="2"/>

</xml_diff>